<commit_message>
Temas_Consultados: nuevo modulo (reemplaza notebook del Tablero); query Athena + clasificacion por categoria + ranking texto para tablero
</commit_message>
<xml_diff>
--- a/Feedback_CES/output/feedback_ces_detalle_mayo_2026.xlsx
+++ b/Feedback_CES/output/feedback_ces_detalle_mayo_2026.xlsx
@@ -1038,7 +1038,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CXF01CUX03 Muy conforme Pushes</t>
+          <t>CXF01CUX03 No sé Pushes</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1058,7 +1058,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CXF01CUX03 No sé Pushes</t>
+          <t>CXF01CUX03 Muy conforme Pushes</t>
         </is>
       </c>
       <c r="B58" t="n">

</xml_diff>